<commit_message>
:kiwi_fruit: LBM dataset 1 (clean datasets)
</commit_message>
<xml_diff>
--- a/data/derived_data/5_SBMclustering/Dataset_1/ps_ITS_rare_expe_D1_tax_table.xlsx
+++ b/data/derived_data/5_SBMclustering/Dataset_1/ps_ITS_rare_expe_D1_tax_table.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="320" uniqueCount="320">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="331" uniqueCount="331">
   <si>
     <t xml:space="preserve"/>
   </si>
@@ -116,12 +116,15 @@
     <t xml:space="preserve">Cluster_105</t>
   </si>
   <si>
+    <t xml:space="preserve">Metschnikowiaceae_105</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Metschnikowia_105</t>
+  </si>
+  <si>
     <t xml:space="preserve">Unknown</t>
   </si>
   <si>
-    <t xml:space="preserve">Unknown_105_105</t>
-  </si>
-  <si>
     <t xml:space="preserve">Cluster_111</t>
   </si>
   <si>
@@ -146,7 +149,13 @@
     <t xml:space="preserve">Cluster_113</t>
   </si>
   <si>
-    <t xml:space="preserve">Unknown_113_113</t>
+    <t xml:space="preserve">Metschnikowiaceae_113</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Metschnikowia_113</t>
+  </si>
+  <si>
+    <t xml:space="preserve">pulcherrima</t>
   </si>
   <si>
     <t xml:space="preserve">Cluster_116</t>
@@ -779,7 +788,10 @@
     <t xml:space="preserve">Cluster_58</t>
   </si>
   <si>
-    <t xml:space="preserve">Unknown_58_58</t>
+    <t xml:space="preserve">Metschnikowiaceae_58</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Metschnikowia_58</t>
   </si>
   <si>
     <t xml:space="preserve">Cluster_59</t>
@@ -809,7 +821,10 @@
     <t xml:space="preserve">Cluster_63</t>
   </si>
   <si>
-    <t xml:space="preserve">Unknown_63_63</t>
+    <t xml:space="preserve">Metschnikowiaceae_63</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Metschnikowia_63</t>
   </si>
   <si>
     <t xml:space="preserve">Cluster_64</t>
@@ -842,7 +857,10 @@
     <t xml:space="preserve">Cluster_68</t>
   </si>
   <si>
-    <t xml:space="preserve">Unknown_68_68</t>
+    <t xml:space="preserve">Metschnikowiaceae_68</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Metschnikowia_68</t>
   </si>
   <si>
     <t xml:space="preserve">Cluster_7</t>
@@ -857,7 +875,10 @@
     <t xml:space="preserve">Cluster_72</t>
   </si>
   <si>
-    <t xml:space="preserve">Unknown_72_72</t>
+    <t xml:space="preserve">Metschnikowiaceae_72</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Metschnikowia_72</t>
   </si>
   <si>
     <t xml:space="preserve">Cluster_73</t>
@@ -902,13 +923,19 @@
     <t xml:space="preserve">Cluster_83</t>
   </si>
   <si>
-    <t xml:space="preserve">Unknown_83_83</t>
+    <t xml:space="preserve">Metschnikowiaceae_83</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Metschnikowia_83</t>
   </si>
   <si>
     <t xml:space="preserve">Cluster_87</t>
   </si>
   <si>
-    <t xml:space="preserve">Unknown_87_87</t>
+    <t xml:space="preserve">Metschnikowiaceae_87</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Metschnikowia_87</t>
   </si>
   <si>
     <t xml:space="preserve">Cluster_88</t>
@@ -920,7 +947,10 @@
     <t xml:space="preserve">Cluster_89</t>
   </si>
   <si>
-    <t xml:space="preserve">Unknown_89_89</t>
+    <t xml:space="preserve">Metschnikowiaceae_89</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Metschnikowia_89</t>
   </si>
   <si>
     <t xml:space="preserve">Cluster_9</t>
@@ -953,7 +983,10 @@
     <t xml:space="preserve">Cluster_95</t>
   </si>
   <si>
-    <t xml:space="preserve">Unknown_95_95</t>
+    <t xml:space="preserve">Metschnikowiaceae_95</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Metschnikowia_95</t>
   </si>
   <si>
     <t xml:space="preserve">Cluster_96</t>
@@ -1435,30 +1468,30 @@
         <v>33</v>
       </c>
       <c r="B6" t="s">
+        <v>9</v>
+      </c>
+      <c r="C6" t="s">
+        <v>10</v>
+      </c>
+      <c r="D6" t="s">
+        <v>11</v>
+      </c>
+      <c r="E6" t="s">
+        <v>17</v>
+      </c>
+      <c r="F6" t="s">
         <v>34</v>
-      </c>
-      <c r="C6" t="s">
-        <v>34</v>
-      </c>
-      <c r="D6" t="s">
-        <v>34</v>
-      </c>
-      <c r="E6" t="s">
-        <v>34</v>
-      </c>
-      <c r="F6" t="s">
-        <v>35</v>
       </c>
       <c r="G6" t="s">
         <v>35</v>
       </c>
       <c r="H6" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B7" t="s">
         <v>9</v>
@@ -1473,18 +1506,18 @@
         <v>17</v>
       </c>
       <c r="F7" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="G7" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="H7" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B8" t="s">
         <v>9</v>
@@ -1499,44 +1532,44 @@
         <v>17</v>
       </c>
       <c r="F8" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="G8" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="H8" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B9" t="s">
-        <v>34</v>
+        <v>9</v>
       </c>
       <c r="C9" t="s">
-        <v>34</v>
+        <v>10</v>
       </c>
       <c r="D9" t="s">
-        <v>34</v>
+        <v>11</v>
       </c>
       <c r="E9" t="s">
-        <v>34</v>
+        <v>17</v>
       </c>
       <c r="F9" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="G9" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="H9" t="s">
-        <v>34</v>
+        <v>47</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="B10" t="s">
         <v>9</v>
@@ -1551,18 +1584,18 @@
         <v>17</v>
       </c>
       <c r="F10" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="G10" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="H10" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="B11" t="s">
         <v>9</v>
@@ -1577,18 +1610,18 @@
         <v>17</v>
       </c>
       <c r="F11" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="G11" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="H11" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="B12" t="s">
         <v>9</v>
@@ -1603,44 +1636,44 @@
         <v>12</v>
       </c>
       <c r="F12" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="G12" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="H12" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="B13" t="s">
         <v>9</v>
       </c>
       <c r="C13" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="D13" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="E13" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="F13" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="G13" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="H13" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="B14" t="s">
         <v>9</v>
@@ -1655,18 +1688,18 @@
         <v>17</v>
       </c>
       <c r="F14" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="G14" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="H14" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="B15" t="s">
         <v>9</v>
@@ -1681,18 +1714,18 @@
         <v>17</v>
       </c>
       <c r="F15" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="G15" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="H15" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="B16" t="s">
         <v>9</v>
@@ -1701,24 +1734,24 @@
         <v>10</v>
       </c>
       <c r="D16" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="E16" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="F16" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="G16" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="H16" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="B17" t="s">
         <v>9</v>
@@ -1730,21 +1763,21 @@
         <v>22</v>
       </c>
       <c r="E17" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="F17" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="G17" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="H17" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="B18" t="s">
         <v>9</v>
@@ -1759,18 +1792,18 @@
         <v>17</v>
       </c>
       <c r="F18" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="G18" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="H18" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="B19" t="s">
         <v>9</v>
@@ -1785,44 +1818,44 @@
         <v>17</v>
       </c>
       <c r="F19" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="G19" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="H19" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="B20" t="s">
         <v>9</v>
       </c>
       <c r="C20" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="D20" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="E20" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="F20" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="G20" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="H20" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="B21" t="s">
         <v>9</v>
@@ -1834,21 +1867,21 @@
         <v>22</v>
       </c>
       <c r="E21" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="F21" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="G21" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="H21" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="B22" t="s">
         <v>9</v>
@@ -1860,47 +1893,47 @@
         <v>22</v>
       </c>
       <c r="E22" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="F22" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="G22" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="H22" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="B23" t="s">
         <v>9</v>
       </c>
       <c r="C23" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="D23" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="E23" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="F23" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="G23" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="H23" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="B24" t="s">
         <v>9</v>
@@ -1912,21 +1945,21 @@
         <v>22</v>
       </c>
       <c r="E24" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="F24" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="G24" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="H24" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="B25" t="s">
         <v>9</v>
@@ -1941,18 +1974,18 @@
         <v>17</v>
       </c>
       <c r="F25" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="G25" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="H25" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="B26" t="s">
         <v>9</v>
@@ -1964,73 +1997,73 @@
         <v>22</v>
       </c>
       <c r="E26" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="F26" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="G26" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="H26" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="B27" t="s">
         <v>9</v>
       </c>
       <c r="C27" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="D27" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="E27" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="F27" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="G27" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="H27" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="B28" t="s">
         <v>9</v>
       </c>
       <c r="C28" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="D28" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="E28" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="F28" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="G28" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="H28" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="B29" t="s">
         <v>9</v>
@@ -2045,44 +2078,44 @@
         <v>29</v>
       </c>
       <c r="F29" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="G29" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="H29" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="B30" t="s">
         <v>9</v>
       </c>
       <c r="C30" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="D30" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="E30" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="F30" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="G30" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="H30" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="B31" t="s">
         <v>9</v>
@@ -2091,24 +2124,24 @@
         <v>10</v>
       </c>
       <c r="D31" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="E31" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="F31" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="G31" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="H31" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="B32" t="s">
         <v>9</v>
@@ -2117,24 +2150,24 @@
         <v>10</v>
       </c>
       <c r="D32" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="E32" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="F32" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="G32" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="H32" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="B33" t="s">
         <v>9</v>
@@ -2149,10 +2182,10 @@
         <v>12</v>
       </c>
       <c r="F33" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="G33" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
       <c r="H33" t="s">
         <v>15</v>
@@ -2160,7 +2193,7 @@
     </row>
     <row r="34">
       <c r="A34" t="s">
-        <v>129</v>
+        <v>132</v>
       </c>
       <c r="B34" t="s">
         <v>9</v>
@@ -2175,70 +2208,70 @@
         <v>17</v>
       </c>
       <c r="F34" t="s">
-        <v>130</v>
+        <v>133</v>
       </c>
       <c r="G34" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="H34" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="B35" t="s">
         <v>9</v>
       </c>
       <c r="C35" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="D35" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="E35" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="F35" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="G35" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="H35" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="B36" t="s">
         <v>9</v>
       </c>
       <c r="C36" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="D36" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="E36" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="F36" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="G36" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="H36" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="B37" t="s">
         <v>9</v>
@@ -2250,21 +2283,21 @@
         <v>22</v>
       </c>
       <c r="E37" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="F37" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="G37" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="H37" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="B38" t="s">
         <v>9</v>
@@ -2279,18 +2312,18 @@
         <v>17</v>
       </c>
       <c r="F38" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="G38" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="H38" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="B39" t="s">
         <v>9</v>
@@ -2302,21 +2335,21 @@
         <v>22</v>
       </c>
       <c r="E39" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="F39" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="G39" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="H39" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="B40" t="s">
         <v>9</v>
@@ -2331,44 +2364,44 @@
         <v>17</v>
       </c>
       <c r="F40" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="G40" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="H40" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="B41" t="s">
         <v>9</v>
       </c>
       <c r="C41" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="D41" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="E41" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="F41" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="G41" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="H41" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="B42" t="s">
         <v>9</v>
@@ -2383,18 +2416,18 @@
         <v>17</v>
       </c>
       <c r="F42" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="G42" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="H42" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="B43" t="s">
         <v>9</v>
@@ -2409,18 +2442,18 @@
         <v>17</v>
       </c>
       <c r="F43" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
       <c r="G43" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="H43" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="B44" t="s">
         <v>9</v>
@@ -2435,18 +2468,18 @@
         <v>17</v>
       </c>
       <c r="F44" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="G44" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="H44" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="B45" t="s">
         <v>9</v>
@@ -2461,10 +2494,10 @@
         <v>29</v>
       </c>
       <c r="F45" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="G45" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="H45" t="s">
         <v>32</v>
@@ -2472,7 +2505,7 @@
     </row>
     <row r="46">
       <c r="A46" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="B46" t="s">
         <v>9</v>
@@ -2484,21 +2517,21 @@
         <v>22</v>
       </c>
       <c r="E46" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="F46" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="G46" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="H46" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="B47" t="s">
         <v>9</v>
@@ -2513,18 +2546,18 @@
         <v>12</v>
       </c>
       <c r="F47" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="G47" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
       <c r="H47" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
       <c r="B48" t="s">
         <v>9</v>
@@ -2533,24 +2566,24 @@
         <v>10</v>
       </c>
       <c r="D48" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="E48" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="F48" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="G48" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="H48" t="s">
-        <v>179</v>
+        <v>182</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
       <c r="B49" t="s">
         <v>9</v>
@@ -2565,18 +2598,18 @@
         <v>17</v>
       </c>
       <c r="F49" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="G49" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
       <c r="H49" t="s">
-        <v>183</v>
+        <v>186</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
       <c r="B50" t="s">
         <v>9</v>
@@ -2591,18 +2624,18 @@
         <v>17</v>
       </c>
       <c r="F50" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
       <c r="G50" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="H50" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="s">
-        <v>187</v>
+        <v>190</v>
       </c>
       <c r="B51" t="s">
         <v>9</v>
@@ -2617,18 +2650,18 @@
         <v>17</v>
       </c>
       <c r="F51" t="s">
-        <v>188</v>
+        <v>191</v>
       </c>
       <c r="G51" t="s">
-        <v>189</v>
+        <v>192</v>
       </c>
       <c r="H51" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="s">
-        <v>190</v>
+        <v>193</v>
       </c>
       <c r="B52" t="s">
         <v>9</v>
@@ -2643,18 +2676,18 @@
         <v>29</v>
       </c>
       <c r="F52" t="s">
-        <v>191</v>
+        <v>194</v>
       </c>
       <c r="G52" t="s">
-        <v>191</v>
+        <v>194</v>
       </c>
       <c r="H52" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="s">
-        <v>192</v>
+        <v>195</v>
       </c>
       <c r="B53" t="s">
         <v>9</v>
@@ -2666,21 +2699,21 @@
         <v>22</v>
       </c>
       <c r="E53" t="s">
-        <v>193</v>
+        <v>196</v>
       </c>
       <c r="F53" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="G53" t="s">
-        <v>195</v>
+        <v>198</v>
       </c>
       <c r="H53" t="s">
-        <v>196</v>
+        <v>199</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="s">
-        <v>197</v>
+        <v>200</v>
       </c>
       <c r="B54" t="s">
         <v>9</v>
@@ -2695,18 +2728,18 @@
         <v>17</v>
       </c>
       <c r="F54" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
       <c r="G54" t="s">
-        <v>199</v>
+        <v>202</v>
       </c>
       <c r="H54" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="s">
-        <v>200</v>
+        <v>203</v>
       </c>
       <c r="B55" t="s">
         <v>9</v>
@@ -2721,18 +2754,18 @@
         <v>17</v>
       </c>
       <c r="F55" t="s">
-        <v>201</v>
+        <v>204</v>
       </c>
       <c r="G55" t="s">
-        <v>202</v>
+        <v>205</v>
       </c>
       <c r="H55" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="s">
-        <v>203</v>
+        <v>206</v>
       </c>
       <c r="B56" t="s">
         <v>9</v>
@@ -2747,10 +2780,10 @@
         <v>17</v>
       </c>
       <c r="F56" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
       <c r="G56" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
       <c r="H56" t="s">
         <v>20</v>
@@ -2758,7 +2791,7 @@
     </row>
     <row r="57">
       <c r="A57" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="B57" t="s">
         <v>9</v>
@@ -2773,18 +2806,18 @@
         <v>17</v>
       </c>
       <c r="F57" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="G57" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
       <c r="H57" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="s">
-        <v>209</v>
+        <v>212</v>
       </c>
       <c r="B58" t="s">
         <v>9</v>
@@ -2799,10 +2832,10 @@
         <v>29</v>
       </c>
       <c r="F58" t="s">
-        <v>210</v>
+        <v>213</v>
       </c>
       <c r="G58" t="s">
-        <v>211</v>
+        <v>214</v>
       </c>
       <c r="H58" t="s">
         <v>32</v>
@@ -2810,33 +2843,33 @@
     </row>
     <row r="59">
       <c r="A59" t="s">
-        <v>212</v>
+        <v>215</v>
       </c>
       <c r="B59" t="s">
         <v>9</v>
       </c>
       <c r="C59" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="D59" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="E59" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="F59" t="s">
-        <v>213</v>
+        <v>216</v>
       </c>
       <c r="G59" t="s">
-        <v>213</v>
+        <v>216</v>
       </c>
       <c r="H59" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="s">
-        <v>214</v>
+        <v>217</v>
       </c>
       <c r="B60" t="s">
         <v>9</v>
@@ -2845,50 +2878,50 @@
         <v>10</v>
       </c>
       <c r="D60" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
       <c r="E60" t="s">
-        <v>216</v>
+        <v>219</v>
       </c>
       <c r="F60" t="s">
-        <v>217</v>
+        <v>220</v>
       </c>
       <c r="G60" t="s">
-        <v>218</v>
+        <v>221</v>
       </c>
       <c r="H60" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="s">
-        <v>219</v>
+        <v>222</v>
       </c>
       <c r="B61" t="s">
         <v>9</v>
       </c>
       <c r="C61" t="s">
-        <v>220</v>
+        <v>223</v>
       </c>
       <c r="D61" t="s">
-        <v>221</v>
+        <v>224</v>
       </c>
       <c r="E61" t="s">
-        <v>222</v>
+        <v>225</v>
       </c>
       <c r="F61" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
       <c r="G61" t="s">
-        <v>224</v>
+        <v>227</v>
       </c>
       <c r="H61" t="s">
-        <v>225</v>
+        <v>228</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="s">
-        <v>226</v>
+        <v>229</v>
       </c>
       <c r="B62" t="s">
         <v>9</v>
@@ -2903,10 +2936,10 @@
         <v>29</v>
       </c>
       <c r="F62" t="s">
-        <v>227</v>
+        <v>230</v>
       </c>
       <c r="G62" t="s">
-        <v>228</v>
+        <v>231</v>
       </c>
       <c r="H62" t="s">
         <v>32</v>
@@ -2914,7 +2947,7 @@
     </row>
     <row r="63">
       <c r="A63" t="s">
-        <v>229</v>
+        <v>232</v>
       </c>
       <c r="B63" t="s">
         <v>9</v>
@@ -2929,44 +2962,44 @@
         <v>17</v>
       </c>
       <c r="F63" t="s">
-        <v>230</v>
+        <v>233</v>
       </c>
       <c r="G63" t="s">
-        <v>231</v>
+        <v>234</v>
       </c>
       <c r="H63" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="s">
-        <v>232</v>
+        <v>235</v>
       </c>
       <c r="B64" t="s">
         <v>9</v>
       </c>
       <c r="C64" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="D64" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="E64" t="s">
-        <v>233</v>
+        <v>236</v>
       </c>
       <c r="F64" t="s">
-        <v>234</v>
+        <v>237</v>
       </c>
       <c r="G64" t="s">
-        <v>235</v>
+        <v>238</v>
       </c>
       <c r="H64" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="s">
-        <v>237</v>
+        <v>240</v>
       </c>
       <c r="B65" t="s">
         <v>9</v>
@@ -2978,47 +3011,47 @@
         <v>22</v>
       </c>
       <c r="E65" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="F65" t="s">
-        <v>238</v>
+        <v>241</v>
       </c>
       <c r="G65" t="s">
-        <v>239</v>
+        <v>242</v>
       </c>
       <c r="H65" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="s">
-        <v>240</v>
+        <v>243</v>
       </c>
       <c r="B66" t="s">
         <v>9</v>
       </c>
       <c r="C66" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="D66" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="E66" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="F66" t="s">
-        <v>241</v>
+        <v>244</v>
       </c>
       <c r="G66" t="s">
-        <v>241</v>
+        <v>244</v>
       </c>
       <c r="H66" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
       <c r="B67" t="s">
         <v>9</v>
@@ -3033,18 +3066,18 @@
         <v>17</v>
       </c>
       <c r="F67" t="s">
-        <v>243</v>
+        <v>246</v>
       </c>
       <c r="G67" t="s">
-        <v>244</v>
+        <v>247</v>
       </c>
       <c r="H67" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
       <c r="B68" t="s">
         <v>9</v>
@@ -3059,18 +3092,18 @@
         <v>17</v>
       </c>
       <c r="F68" t="s">
-        <v>246</v>
+        <v>249</v>
       </c>
       <c r="G68" t="s">
-        <v>247</v>
+        <v>250</v>
       </c>
       <c r="H68" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="B69" t="s">
         <v>9</v>
@@ -3085,18 +3118,18 @@
         <v>17</v>
       </c>
       <c r="F69" t="s">
-        <v>249</v>
+        <v>252</v>
       </c>
       <c r="G69" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
       <c r="H69" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
       <c r="B70" t="s">
         <v>9</v>
@@ -3111,44 +3144,44 @@
         <v>17</v>
       </c>
       <c r="F70" t="s">
-        <v>252</v>
+        <v>255</v>
       </c>
       <c r="G70" t="s">
-        <v>253</v>
+        <v>256</v>
       </c>
       <c r="H70" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="s">
-        <v>254</v>
+        <v>257</v>
       </c>
       <c r="B71" t="s">
-        <v>34</v>
+        <v>9</v>
       </c>
       <c r="C71" t="s">
-        <v>34</v>
+        <v>10</v>
       </c>
       <c r="D71" t="s">
-        <v>34</v>
+        <v>11</v>
       </c>
       <c r="E71" t="s">
-        <v>34</v>
+        <v>17</v>
       </c>
       <c r="F71" t="s">
-        <v>255</v>
+        <v>258</v>
       </c>
       <c r="G71" t="s">
-        <v>255</v>
+        <v>259</v>
       </c>
       <c r="H71" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="s">
-        <v>256</v>
+        <v>260</v>
       </c>
       <c r="B72" t="s">
         <v>9</v>
@@ -3163,18 +3196,18 @@
         <v>17</v>
       </c>
       <c r="F72" t="s">
-        <v>257</v>
+        <v>261</v>
       </c>
       <c r="G72" t="s">
-        <v>258</v>
+        <v>262</v>
       </c>
       <c r="H72" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="s">
-        <v>259</v>
+        <v>263</v>
       </c>
       <c r="B73" t="s">
         <v>9</v>
@@ -3183,76 +3216,76 @@
         <v>10</v>
       </c>
       <c r="D73" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
       <c r="E73" t="s">
-        <v>216</v>
+        <v>219</v>
       </c>
       <c r="F73" t="s">
-        <v>260</v>
+        <v>264</v>
       </c>
       <c r="G73" t="s">
-        <v>261</v>
+        <v>265</v>
       </c>
       <c r="H73" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="s">
-        <v>262</v>
+        <v>266</v>
       </c>
       <c r="B74" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C74" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="D74" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="E74" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="F74" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="G74" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="H74" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="s">
-        <v>264</v>
+        <v>268</v>
       </c>
       <c r="B75" t="s">
-        <v>34</v>
+        <v>9</v>
       </c>
       <c r="C75" t="s">
-        <v>34</v>
+        <v>10</v>
       </c>
       <c r="D75" t="s">
-        <v>34</v>
+        <v>11</v>
       </c>
       <c r="E75" t="s">
-        <v>34</v>
+        <v>17</v>
       </c>
       <c r="F75" t="s">
-        <v>265</v>
+        <v>269</v>
       </c>
       <c r="G75" t="s">
-        <v>265</v>
+        <v>270</v>
       </c>
       <c r="H75" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="s">
-        <v>266</v>
+        <v>271</v>
       </c>
       <c r="B76" t="s">
         <v>9</v>
@@ -3267,44 +3300,44 @@
         <v>17</v>
       </c>
       <c r="F76" t="s">
-        <v>267</v>
+        <v>272</v>
       </c>
       <c r="G76" t="s">
-        <v>268</v>
+        <v>273</v>
       </c>
       <c r="H76" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="s">
-        <v>269</v>
+        <v>274</v>
       </c>
       <c r="B77" t="s">
         <v>9</v>
       </c>
       <c r="C77" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="D77" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="E77" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="F77" t="s">
-        <v>270</v>
+        <v>275</v>
       </c>
       <c r="G77" t="s">
-        <v>270</v>
+        <v>275</v>
       </c>
       <c r="H77" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="s">
-        <v>271</v>
+        <v>276</v>
       </c>
       <c r="B78" t="s">
         <v>9</v>
@@ -3319,44 +3352,44 @@
         <v>17</v>
       </c>
       <c r="F78" t="s">
-        <v>272</v>
+        <v>277</v>
       </c>
       <c r="G78" t="s">
-        <v>273</v>
+        <v>278</v>
       </c>
       <c r="H78" t="s">
-        <v>274</v>
+        <v>279</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="s">
-        <v>275</v>
+        <v>280</v>
       </c>
       <c r="B79" t="s">
-        <v>34</v>
+        <v>9</v>
       </c>
       <c r="C79" t="s">
-        <v>34</v>
+        <v>10</v>
       </c>
       <c r="D79" t="s">
-        <v>34</v>
+        <v>11</v>
       </c>
       <c r="E79" t="s">
-        <v>34</v>
+        <v>17</v>
       </c>
       <c r="F79" t="s">
-        <v>276</v>
+        <v>281</v>
       </c>
       <c r="G79" t="s">
-        <v>276</v>
+        <v>282</v>
       </c>
       <c r="H79" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="s">
-        <v>277</v>
+        <v>283</v>
       </c>
       <c r="B80" t="s">
         <v>9</v>
@@ -3371,44 +3404,44 @@
         <v>29</v>
       </c>
       <c r="F80" t="s">
-        <v>278</v>
+        <v>284</v>
       </c>
       <c r="G80" t="s">
-        <v>279</v>
+        <v>285</v>
       </c>
       <c r="H80" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="s">
-        <v>280</v>
+        <v>286</v>
       </c>
       <c r="B81" t="s">
-        <v>34</v>
+        <v>9</v>
       </c>
       <c r="C81" t="s">
-        <v>34</v>
+        <v>10</v>
       </c>
       <c r="D81" t="s">
-        <v>34</v>
+        <v>11</v>
       </c>
       <c r="E81" t="s">
-        <v>34</v>
+        <v>17</v>
       </c>
       <c r="F81" t="s">
-        <v>281</v>
+        <v>287</v>
       </c>
       <c r="G81" t="s">
-        <v>281</v>
+        <v>288</v>
       </c>
       <c r="H81" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="s">
-        <v>282</v>
+        <v>289</v>
       </c>
       <c r="B82" t="s">
         <v>9</v>
@@ -3423,18 +3456,18 @@
         <v>17</v>
       </c>
       <c r="F82" t="s">
-        <v>283</v>
+        <v>290</v>
       </c>
       <c r="G82" t="s">
-        <v>284</v>
+        <v>291</v>
       </c>
       <c r="H82" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="s">
-        <v>285</v>
+        <v>292</v>
       </c>
       <c r="B83" t="s">
         <v>9</v>
@@ -3449,18 +3482,18 @@
         <v>17</v>
       </c>
       <c r="F83" t="s">
-        <v>286</v>
+        <v>293</v>
       </c>
       <c r="G83" t="s">
-        <v>287</v>
+        <v>294</v>
       </c>
       <c r="H83" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="s">
-        <v>288</v>
+        <v>295</v>
       </c>
       <c r="B84" t="s">
         <v>9</v>
@@ -3475,18 +3508,18 @@
         <v>23</v>
       </c>
       <c r="F84" t="s">
-        <v>289</v>
+        <v>296</v>
       </c>
       <c r="G84" t="s">
-        <v>290</v>
+        <v>297</v>
       </c>
       <c r="H84" t="s">
-        <v>291</v>
+        <v>298</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="s">
-        <v>292</v>
+        <v>299</v>
       </c>
       <c r="B85" t="s">
         <v>9</v>
@@ -3501,70 +3534,70 @@
         <v>17</v>
       </c>
       <c r="F85" t="s">
-        <v>293</v>
+        <v>300</v>
       </c>
       <c r="G85" t="s">
-        <v>294</v>
+        <v>301</v>
       </c>
       <c r="H85" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="s">
-        <v>295</v>
+        <v>302</v>
       </c>
       <c r="B86" t="s">
-        <v>34</v>
+        <v>9</v>
       </c>
       <c r="C86" t="s">
-        <v>34</v>
+        <v>10</v>
       </c>
       <c r="D86" t="s">
-        <v>34</v>
+        <v>11</v>
       </c>
       <c r="E86" t="s">
-        <v>34</v>
+        <v>17</v>
       </c>
       <c r="F86" t="s">
-        <v>296</v>
+        <v>303</v>
       </c>
       <c r="G86" t="s">
-        <v>296</v>
+        <v>304</v>
       </c>
       <c r="H86" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="s">
-        <v>297</v>
+        <v>305</v>
       </c>
       <c r="B87" t="s">
-        <v>34</v>
+        <v>9</v>
       </c>
       <c r="C87" t="s">
-        <v>34</v>
+        <v>10</v>
       </c>
       <c r="D87" t="s">
-        <v>34</v>
+        <v>11</v>
       </c>
       <c r="E87" t="s">
-        <v>34</v>
+        <v>17</v>
       </c>
       <c r="F87" t="s">
-        <v>298</v>
+        <v>306</v>
       </c>
       <c r="G87" t="s">
-        <v>298</v>
+        <v>307</v>
       </c>
       <c r="H87" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="s">
-        <v>299</v>
+        <v>308</v>
       </c>
       <c r="B88" t="s">
         <v>9</v>
@@ -3579,44 +3612,44 @@
         <v>29</v>
       </c>
       <c r="F88" t="s">
-        <v>300</v>
+        <v>309</v>
       </c>
       <c r="G88" t="s">
-        <v>300</v>
+        <v>309</v>
       </c>
       <c r="H88" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="s">
-        <v>301</v>
+        <v>310</v>
       </c>
       <c r="B89" t="s">
-        <v>34</v>
+        <v>9</v>
       </c>
       <c r="C89" t="s">
-        <v>34</v>
+        <v>10</v>
       </c>
       <c r="D89" t="s">
-        <v>34</v>
+        <v>11</v>
       </c>
       <c r="E89" t="s">
-        <v>34</v>
+        <v>17</v>
       </c>
       <c r="F89" t="s">
-        <v>302</v>
+        <v>311</v>
       </c>
       <c r="G89" t="s">
-        <v>302</v>
+        <v>312</v>
       </c>
       <c r="H89" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="s">
-        <v>303</v>
+        <v>313</v>
       </c>
       <c r="B90" t="s">
         <v>9</v>
@@ -3631,18 +3664,18 @@
         <v>17</v>
       </c>
       <c r="F90" t="s">
-        <v>304</v>
+        <v>314</v>
       </c>
       <c r="G90" t="s">
-        <v>305</v>
+        <v>315</v>
       </c>
       <c r="H90" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="s">
-        <v>306</v>
+        <v>316</v>
       </c>
       <c r="B91" t="s">
         <v>9</v>
@@ -3657,18 +3690,18 @@
         <v>29</v>
       </c>
       <c r="F91" t="s">
-        <v>307</v>
+        <v>317</v>
       </c>
       <c r="G91" t="s">
-        <v>308</v>
+        <v>318</v>
       </c>
       <c r="H91" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="s">
-        <v>309</v>
+        <v>319</v>
       </c>
       <c r="B92" t="s">
         <v>9</v>
@@ -3683,44 +3716,44 @@
         <v>17</v>
       </c>
       <c r="F92" t="s">
-        <v>310</v>
+        <v>320</v>
       </c>
       <c r="G92" t="s">
-        <v>311</v>
+        <v>321</v>
       </c>
       <c r="H92" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="s">
-        <v>312</v>
+        <v>322</v>
       </c>
       <c r="B93" t="s">
-        <v>34</v>
+        <v>9</v>
       </c>
       <c r="C93" t="s">
-        <v>34</v>
+        <v>10</v>
       </c>
       <c r="D93" t="s">
-        <v>34</v>
+        <v>11</v>
       </c>
       <c r="E93" t="s">
-        <v>34</v>
+        <v>17</v>
       </c>
       <c r="F93" t="s">
-        <v>313</v>
+        <v>323</v>
       </c>
       <c r="G93" t="s">
-        <v>313</v>
+        <v>324</v>
       </c>
       <c r="H93" t="s">
-        <v>34</v>
+        <v>47</v>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="s">
-        <v>314</v>
+        <v>325</v>
       </c>
       <c r="B94" t="s">
         <v>9</v>
@@ -3735,18 +3768,18 @@
         <v>17</v>
       </c>
       <c r="F94" t="s">
-        <v>315</v>
+        <v>326</v>
       </c>
       <c r="G94" t="s">
-        <v>316</v>
+        <v>327</v>
       </c>
       <c r="H94" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="s">
-        <v>317</v>
+        <v>328</v>
       </c>
       <c r="B95" t="s">
         <v>9</v>
@@ -3758,16 +3791,16 @@
         <v>22</v>
       </c>
       <c r="E95" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="F95" t="s">
-        <v>318</v>
+        <v>329</v>
       </c>
       <c r="G95" t="s">
-        <v>319</v>
+        <v>330</v>
       </c>
       <c r="H95" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
     </row>
   </sheetData>

</xml_diff>